<commit_message>
fix(catalog): explain existing tag import blocking
</commit_message>
<xml_diff>
--- a/public/templates/plantilla-importacion-catalogo.xlsx
+++ b/public/templates/plantilla-importacion-catalogo.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" r:id="R1160617ec2ca4d92"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listado maestro" sheetId="2" r:id="R5a97081df03c4db2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categorías N4" sheetId="3" r:id="R3c6f18934ef643fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Características" sheetId="4" r:id="Ra3343e06b71e4de6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Especificaciones" sheetId="5" r:id="Ra764f3e5bdbe4069"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fabricantes de referencia" sheetId="6" r:id="R65be4785eeaf4479"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" r:id="R04b29b8c28394ddb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listado maestro" sheetId="2" r:id="R8d9865a126c4422e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categorías N4" sheetId="3" r:id="Rac8b71ab59e84173"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Características" sheetId="4" r:id="R846fa4f881c745af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Especificaciones" sheetId="5" r:id="Rd59f7facf3af4559"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fabricantes de referencia" sheetId="6" r:id="Rf8bd3157ab1c45b4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -996,7 +996,7 @@
     </x:row>
     <x:row r="50" ht="23" customHeight="1">
       <x:c r="A50" s="6" t="str">
-        <x:v>4. Qué ocurre al repetir un TAG</x:v>
+        <x:v>4. TAG existentes: carga bloqueada</x:v>
       </x:c>
       <x:c r="B50" s="6" t="str">
         <x:v>4. Qué ocurre al repetir un TAG</x:v>
@@ -1010,7 +1010,7 @@
     </x:row>
     <x:row r="51" ht="23" customHeight="1">
       <x:c r="A51" s="5" t="str">
-        <x:v>Un TAG existente actualiza su modelo y conserva su foto. Las especificaciones, componentes y redes se reemplazan por los datos del archivo. Si la hoja Fabricantes de referencia está presente, sus filas reemplazan las referencias de los TAG del listado; si un TAG no tiene filas, sus referencias se vacían. Los archivos anteriores sin esa hoja conservan las referencias existentes. Los modelos que no aparecen en Listado maestro se conservan.</x:v>
+        <x:v>Si un TAG de Listado maestro ya existe en el catálogo, se bloquea toda la carga sin guardar cambios. El análisis indica la fila, el TAG y todas sus redes actuales (o que no tiene redes asignadas). Elegir otra red, cambiar el nombre o aceptar modelos sin especificaciones no permite sobrescribirlo. Retira del archivo el TAG existente y sus filas de detalle, y vuelve a analizar. La comprobación se repite al confirmar.</x:v>
       </x:c>
       <x:c r="B51" s="5" t="str">
         <x:v>Un TAG existente actualiza su modelo y conserva su foto. Las especificaciones, componentes y redes se reemplazan por los datos del archivo. Si la hoja Fabricantes de referencia está presente, sus filas reemplazan las referencias de los TAG del listado; si un TAG no tiene filas, sus referencias se vacían. Los archivos anteriores sin esa hoja conservan las referencias existentes. Los modelos que no aparecen en Listado maestro se conservan.</x:v>
@@ -2109,7 +2109,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R6ac328ee3fe14c41"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb77120cc35d4eb8"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2565,7 +2565,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R21728399acdc47c6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5de493a66884779"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2989,7 +2989,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R92db91d8c43d4270"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra851cbc372014af1"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3621,7 +3621,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3867f0af95e84d9d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4157851b7be4fa6"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4253,7 +4253,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf01d4ae9b84142d3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R414609714c204d8d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat(catalog): manage model references and update the Excel template
</commit_message>
<xml_diff>
--- a/public/templates/plantilla-importacion-catalogo.xlsx
+++ b/public/templates/plantilla-importacion-catalogo.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" r:id="R04b29b8c28394ddb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listado maestro" sheetId="2" r:id="R8d9865a126c4422e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categorías N4" sheetId="3" r:id="Rac8b71ab59e84173"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Características" sheetId="4" r:id="R846fa4f881c745af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Especificaciones" sheetId="5" r:id="Rd59f7facf3af4559"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fabricantes de referencia" sheetId="6" r:id="Rf8bd3157ab1c45b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" r:id="R659fecd997c143d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Listado maestro" sheetId="2" r:id="R581d9080fa1f4573"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Categorías N4" sheetId="3" r:id="Rd8a4f6be6da14ad1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Características" sheetId="4" r:id="Ra33fb73a56024184"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Especificaciones" sheetId="5" r:id="R210c55c8224d4548"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fabricantes de referencia" sheetId="6" r:id="Rc354829e9c1e4a6a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -203,16 +203,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ListadoMaestro" displayName="ListadoMaestro" ref="A1:G2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A1:G2"/>
-  <x:tableColumns count="7">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="ListadoMaestro" displayName="ListadoMaestro" ref="A1:F2" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A1:F2"/>
+  <x:tableColumns count="6">
     <x:tableColumn id="1" name="TAG ACTIVO"/>
     <x:tableColumn id="2" name="Nombre"/>
     <x:tableColumn id="3" name="Código CA"/>
     <x:tableColumn id="4" name="Categoría N4"/>
     <x:tableColumn id="5" name="Tipo"/>
-    <x:tableColumn id="6" name="Fabricante / modelo"/>
-    <x:tableColumn id="7" name="Denominación de etapa"/>
+    <x:tableColumn id="6" name="Denominación de etapa"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -577,7 +576,7 @@
         <x:v>Listado maestro</x:v>
       </x:c>
       <x:c r="B10" s="3" t="str">
-        <x:v>Una fila por activo. Completa TAG ACTIVO (único), Nombre, Código CA, Categoría N4, Tipo, Fabricante / modelo y Denominación de etapa. Usa el nombre exacto de una etapa existente en el sistema, por ejemplo Molienda primaria. En Fabricante / modelo usa el fabricante conocido o Pendiente; este campo es independiente de los fabricantes de referencia.</x:v>
+        <x:v>Una fila por activo. Completa TAG ACTIVO (único), Nombre, Código CA, Categoría N4, Tipo y Denominación de etapa. Usa el nombre exacto de una etapa existente en el sistema, por ejemplo Molienda primaria. Los fabricantes se cargan únicamente en Fabricantes de referencia. Si un archivo anterior incluye Fabricante / modelo, esa columna se ignora.</x:v>
       </x:c>
       <x:c r="C10" s="3"/>
       <x:c r="D10" s="3"/>
@@ -647,7 +646,7 @@
         <x:v>Fabricantes de referencia</x:v>
       </x:c>
       <x:c r="B19" s="3" t="str">
-        <x:v>Una fila por fabricante: TAG ACTIVO, Fabricante, Descripción y Sitio web. TAG y Fabricante son obligatorios; Descripción y Sitio web son opcionales. Usa direcciones completas http:// o https://. Repite el TAG para asociar varios fabricantes. Si no hay referencias, no agregues filas para ese activo.</x:v>
+        <x:v>Una fila por fabricante: TAG ACTIVO, Fabricante, Descripción y Sitio web. TAG y Fabricante son obligatorios; Descripción y Sitio web son opcionales. Usa direcciones completas http:// o https://. Repite el TAG para asociar varios fabricantes. Si no hay referencias, no agregues filas para ese activo. Estos nombres alimentan los filtros del catálogo; cada modelo puede tener varios fabricantes.</x:v>
       </x:c>
       <x:c r="C19" s="3"/>
       <x:c r="D19" s="3"/>
@@ -999,69 +998,69 @@
         <x:v>4. TAG existentes: carga bloqueada</x:v>
       </x:c>
       <x:c r="B50" s="6" t="str">
-        <x:v>4. Qué ocurre al repetir un TAG</x:v>
+        <x:v>4. TAG existentes: carga bloqueada</x:v>
       </x:c>
       <x:c r="C50" s="6" t="str">
-        <x:v>4. Qué ocurre al repetir un TAG</x:v>
+        <x:v>4. TAG existentes: carga bloqueada</x:v>
       </x:c>
       <x:c r="D50" s="6" t="str">
-        <x:v>4. Qué ocurre al repetir un TAG</x:v>
+        <x:v>4. TAG existentes: carga bloqueada</x:v>
       </x:c>
     </x:row>
     <x:row r="51" ht="23" customHeight="1">
       <x:c r="A51" s="5" t="str">
-        <x:v>Si un TAG de Listado maestro ya existe en el catálogo, se bloquea toda la carga sin guardar cambios. El análisis indica la fila, el TAG y todas sus redes actuales (o que no tiene redes asignadas). Elegir otra red, cambiar el nombre o aceptar modelos sin especificaciones no permite sobrescribirlo. Retira del archivo el TAG existente y sus filas de detalle, y vuelve a analizar. La comprobación se repite al confirmar.</x:v>
+        <x:v>Si un TAG ya existe en el catálogo, se bloquea toda la carga sin guardar cambios y se indican sus redes actuales. Retira ese TAG y sus filas de detalle antes de analizar nuevamente. Los duplicados por tipo, conjunto de fabricantes de referencia, nombre y etapa requieren aceptar la opción de duplicados con TAG distintos. Sin referencias, se compara el conjunto vacío. Los TAG existentes nunca se sobrescriben.</x:v>
       </x:c>
       <x:c r="B51" s="5" t="str">
-        <x:v>Un TAG existente actualiza su modelo y conserva su foto. Las especificaciones, componentes y redes se reemplazan por los datos del archivo. Si la hoja Fabricantes de referencia está presente, sus filas reemplazan las referencias de los TAG del listado; si un TAG no tiene filas, sus referencias se vacían. Los archivos anteriores sin esa hoja conservan las referencias existentes. Los modelos que no aparecen en Listado maestro se conservan.</x:v>
+        <x:v>Si un TAG ya existe en el catálogo, se bloquea toda la carga sin guardar cambios y se indican sus redes actuales. Retira ese TAG y sus filas de detalle antes de analizar nuevamente. Los duplicados por tipo, conjunto de fabricantes de referencia, nombre y etapa requieren aceptar la opción de duplicados con TAG distintos. Sin referencias, se compara el conjunto vacío. Los TAG existentes nunca se sobrescriben.</x:v>
       </x:c>
       <x:c r="C51" s="5" t="str">
-        <x:v>Un TAG existente actualiza su modelo y conserva su foto. Las especificaciones, componentes y redes se reemplazan por los datos del archivo. Si la hoja Fabricantes de referencia está presente, sus filas reemplazan las referencias de los TAG del listado; si un TAG no tiene filas, sus referencias se vacían. Los archivos anteriores sin esa hoja conservan las referencias existentes. Los modelos que no aparecen en Listado maestro se conservan.</x:v>
+        <x:v>Si un TAG ya existe en el catálogo, se bloquea toda la carga sin guardar cambios y se indican sus redes actuales. Retira ese TAG y sus filas de detalle antes de analizar nuevamente. Los duplicados por tipo, conjunto de fabricantes de referencia, nombre y etapa requieren aceptar la opción de duplicados con TAG distintos. Sin referencias, se compara el conjunto vacío. Los TAG existentes nunca se sobrescriben.</x:v>
       </x:c>
       <x:c r="D51" s="5" t="str">
-        <x:v>Un TAG existente actualiza su modelo y conserva su foto. Las especificaciones, componentes y redes se reemplazan por los datos del archivo. Si la hoja Fabricantes de referencia está presente, sus filas reemplazan las referencias de los TAG del listado; si un TAG no tiene filas, sus referencias se vacían. Los archivos anteriores sin esa hoja conservan las referencias existentes. Los modelos que no aparecen en Listado maestro se conservan.</x:v>
+        <x:v>Si un TAG ya existe en el catálogo, se bloquea toda la carga sin guardar cambios y se indican sus redes actuales. Retira ese TAG y sus filas de detalle antes de analizar nuevamente. Los duplicados por tipo, conjunto de fabricantes de referencia, nombre y etapa requieren aceptar la opción de duplicados con TAG distintos. Sin referencias, se compara el conjunto vacío. Los TAG existentes nunca se sobrescriben.</x:v>
       </x:c>
     </x:row>
     <x:row r="52" ht="23" customHeight="1">
       <x:c r="A52" s="5" t="str">
-        <x:v>Un TAG existente actualiza su modelo y conserva su foto. Las especificaciones, componentes y redes se reemplazan por los datos del archivo. Si la hoja Fabricantes de referencia está presente, sus filas reemplazan las referencias de los TAG del listado; si un TAG no tiene filas, sus referencias se vacían. Los archivos anteriores sin esa hoja conservan las referencias existentes. Los modelos que no aparecen en Listado maestro se conservan.</x:v>
+        <x:v>Si un TAG ya existe en el catálogo, se bloquea toda la carga sin guardar cambios y se indican sus redes actuales. Retira ese TAG y sus filas de detalle antes de analizar nuevamente. Los duplicados por tipo, conjunto de fabricantes de referencia, nombre y etapa requieren aceptar la opción de duplicados con TAG distintos. Sin referencias, se compara el conjunto vacío. Los TAG existentes nunca se sobrescriben.</x:v>
       </x:c>
       <x:c r="B52" s="5" t="str">
-        <x:v>Un TAG existente actualiza su modelo y conserva su foto. Las especificaciones, componentes y redes se reemplazan por los datos del archivo. Si la hoja Fabricantes de referencia está presente, sus filas reemplazan las referencias de los TAG del listado; si un TAG no tiene filas, sus referencias se vacían. Los archivos anteriores sin esa hoja conservan las referencias existentes. Los modelos que no aparecen en Listado maestro se conservan.</x:v>
+        <x:v>Si un TAG ya existe en el catálogo, se bloquea toda la carga sin guardar cambios y se indican sus redes actuales. Retira ese TAG y sus filas de detalle antes de analizar nuevamente. Los duplicados por tipo, conjunto de fabricantes de referencia, nombre y etapa requieren aceptar la opción de duplicados con TAG distintos. Sin referencias, se compara el conjunto vacío. Los TAG existentes nunca se sobrescriben.</x:v>
       </x:c>
       <x:c r="C52" s="5" t="str">
-        <x:v>Un TAG existente actualiza su modelo y conserva su foto. Las especificaciones, componentes y redes se reemplazan por los datos del archivo. Si la hoja Fabricantes de referencia está presente, sus filas reemplazan las referencias de los TAG del listado; si un TAG no tiene filas, sus referencias se vacían. Los archivos anteriores sin esa hoja conservan las referencias existentes. Los modelos que no aparecen en Listado maestro se conservan.</x:v>
+        <x:v>Si un TAG ya existe en el catálogo, se bloquea toda la carga sin guardar cambios y se indican sus redes actuales. Retira ese TAG y sus filas de detalle antes de analizar nuevamente. Los duplicados por tipo, conjunto de fabricantes de referencia, nombre y etapa requieren aceptar la opción de duplicados con TAG distintos. Sin referencias, se compara el conjunto vacío. Los TAG existentes nunca se sobrescriben.</x:v>
       </x:c>
       <x:c r="D52" s="5" t="str">
-        <x:v>Un TAG existente actualiza su modelo y conserva su foto. Las especificaciones, componentes y redes se reemplazan por los datos del archivo. Si la hoja Fabricantes de referencia está presente, sus filas reemplazan las referencias de los TAG del listado; si un TAG no tiene filas, sus referencias se vacían. Los archivos anteriores sin esa hoja conservan las referencias existentes. Los modelos que no aparecen en Listado maestro se conservan.</x:v>
+        <x:v>Si un TAG ya existe en el catálogo, se bloquea toda la carga sin guardar cambios y se indican sus redes actuales. Retira ese TAG y sus filas de detalle antes de analizar nuevamente. Los duplicados por tipo, conjunto de fabricantes de referencia, nombre y etapa requieren aceptar la opción de duplicados con TAG distintos. Sin referencias, se compara el conjunto vacío. Los TAG existentes nunca se sobrescriben.</x:v>
       </x:c>
     </x:row>
     <x:row r="53" ht="23" customHeight="1">
       <x:c r="A53" s="5" t="str">
-        <x:v>Un TAG existente actualiza su modelo y conserva su foto. Las especificaciones, componentes y redes se reemplazan por los datos del archivo. Si la hoja Fabricantes de referencia está presente, sus filas reemplazan las referencias de los TAG del listado; si un TAG no tiene filas, sus referencias se vacían. Los archivos anteriores sin esa hoja conservan las referencias existentes. Los modelos que no aparecen en Listado maestro se conservan.</x:v>
+        <x:v>Si un TAG ya existe en el catálogo, se bloquea toda la carga sin guardar cambios y se indican sus redes actuales. Retira ese TAG y sus filas de detalle antes de analizar nuevamente. Los duplicados por tipo, conjunto de fabricantes de referencia, nombre y etapa requieren aceptar la opción de duplicados con TAG distintos. Sin referencias, se compara el conjunto vacío. Los TAG existentes nunca se sobrescriben.</x:v>
       </x:c>
       <x:c r="B53" s="5" t="str">
-        <x:v>Un TAG existente actualiza su modelo y conserva su foto. Las especificaciones, componentes y redes se reemplazan por los datos del archivo. Si la hoja Fabricantes de referencia está presente, sus filas reemplazan las referencias de los TAG del listado; si un TAG no tiene filas, sus referencias se vacían. Los archivos anteriores sin esa hoja conservan las referencias existentes. Los modelos que no aparecen en Listado maestro se conservan.</x:v>
+        <x:v>Si un TAG ya existe en el catálogo, se bloquea toda la carga sin guardar cambios y se indican sus redes actuales. Retira ese TAG y sus filas de detalle antes de analizar nuevamente. Los duplicados por tipo, conjunto de fabricantes de referencia, nombre y etapa requieren aceptar la opción de duplicados con TAG distintos. Sin referencias, se compara el conjunto vacío. Los TAG existentes nunca se sobrescriben.</x:v>
       </x:c>
       <x:c r="C53" s="5" t="str">
-        <x:v>Un TAG existente actualiza su modelo y conserva su foto. Las especificaciones, componentes y redes se reemplazan por los datos del archivo. Si la hoja Fabricantes de referencia está presente, sus filas reemplazan las referencias de los TAG del listado; si un TAG no tiene filas, sus referencias se vacían. Los archivos anteriores sin esa hoja conservan las referencias existentes. Los modelos que no aparecen en Listado maestro se conservan.</x:v>
+        <x:v>Si un TAG ya existe en el catálogo, se bloquea toda la carga sin guardar cambios y se indican sus redes actuales. Retira ese TAG y sus filas de detalle antes de analizar nuevamente. Los duplicados por tipo, conjunto de fabricantes de referencia, nombre y etapa requieren aceptar la opción de duplicados con TAG distintos. Sin referencias, se compara el conjunto vacío. Los TAG existentes nunca se sobrescriben.</x:v>
       </x:c>
       <x:c r="D53" s="5" t="str">
-        <x:v>Un TAG existente actualiza su modelo y conserva su foto. Las especificaciones, componentes y redes se reemplazan por los datos del archivo. Si la hoja Fabricantes de referencia está presente, sus filas reemplazan las referencias de los TAG del listado; si un TAG no tiene filas, sus referencias se vacían. Los archivos anteriores sin esa hoja conservan las referencias existentes. Los modelos que no aparecen en Listado maestro se conservan.</x:v>
+        <x:v>Si un TAG ya existe en el catálogo, se bloquea toda la carga sin guardar cambios y se indican sus redes actuales. Retira ese TAG y sus filas de detalle antes de analizar nuevamente. Los duplicados por tipo, conjunto de fabricantes de referencia, nombre y etapa requieren aceptar la opción de duplicados con TAG distintos. Sin referencias, se compara el conjunto vacío. Los TAG existentes nunca se sobrescriben.</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="23" customHeight="1">
       <x:c r="A54" s="5" t="str">
-        <x:v>Un TAG existente actualiza su modelo y conserva su foto. Las especificaciones, componentes y redes se reemplazan por los datos del archivo. Si la hoja Fabricantes de referencia está presente, sus filas reemplazan las referencias de los TAG del listado; si un TAG no tiene filas, sus referencias se vacían. Los archivos anteriores sin esa hoja conservan las referencias existentes. Los modelos que no aparecen en Listado maestro se conservan.</x:v>
+        <x:v>Si un TAG ya existe en el catálogo, se bloquea toda la carga sin guardar cambios y se indican sus redes actuales. Retira ese TAG y sus filas de detalle antes de analizar nuevamente. Los duplicados por tipo, conjunto de fabricantes de referencia, nombre y etapa requieren aceptar la opción de duplicados con TAG distintos. Sin referencias, se compara el conjunto vacío. Los TAG existentes nunca se sobrescriben.</x:v>
       </x:c>
       <x:c r="B54" s="5" t="str">
-        <x:v>Un TAG existente actualiza su modelo y conserva su foto. Las especificaciones, componentes y redes se reemplazan por los datos del archivo. Si la hoja Fabricantes de referencia está presente, sus filas reemplazan las referencias de los TAG del listado; si un TAG no tiene filas, sus referencias se vacían. Los archivos anteriores sin esa hoja conservan las referencias existentes. Los modelos que no aparecen en Listado maestro se conservan.</x:v>
+        <x:v>Si un TAG ya existe en el catálogo, se bloquea toda la carga sin guardar cambios y se indican sus redes actuales. Retira ese TAG y sus filas de detalle antes de analizar nuevamente. Los duplicados por tipo, conjunto de fabricantes de referencia, nombre y etapa requieren aceptar la opción de duplicados con TAG distintos. Sin referencias, se compara el conjunto vacío. Los TAG existentes nunca se sobrescriben.</x:v>
       </x:c>
       <x:c r="C54" s="5" t="str">
-        <x:v>Un TAG existente actualiza su modelo y conserva su foto. Las especificaciones, componentes y redes se reemplazan por los datos del archivo. Si la hoja Fabricantes de referencia está presente, sus filas reemplazan las referencias de los TAG del listado; si un TAG no tiene filas, sus referencias se vacían. Los archivos anteriores sin esa hoja conservan las referencias existentes. Los modelos que no aparecen en Listado maestro se conservan.</x:v>
+        <x:v>Si un TAG ya existe en el catálogo, se bloquea toda la carga sin guardar cambios y se indican sus redes actuales. Retira ese TAG y sus filas de detalle antes de analizar nuevamente. Los duplicados por tipo, conjunto de fabricantes de referencia, nombre y etapa requieren aceptar la opción de duplicados con TAG distintos. Sin referencias, se compara el conjunto vacío. Los TAG existentes nunca se sobrescriben.</x:v>
       </x:c>
       <x:c r="D54" s="5" t="str">
-        <x:v>Un TAG existente actualiza su modelo y conserva su foto. Las especificaciones, componentes y redes se reemplazan por los datos del archivo. Si la hoja Fabricantes de referencia está presente, sus filas reemplazan las referencias de los TAG del listado; si un TAG no tiene filas, sus referencias se vacían. Los archivos anteriores sin esa hoja conservan las referencias existentes. Los modelos que no aparecen en Listado maestro se conservan.</x:v>
+        <x:v>Si un TAG ya existe en el catálogo, se bloquea toda la carga sin guardar cambios y se indican sus redes actuales. Retira ese TAG y sus filas de detalle antes de analizar nuevamente. Los duplicados por tipo, conjunto de fabricantes de referencia, nombre y etapa requieren aceptar la opción de duplicados con TAG distintos. Sin referencias, se compara el conjunto vacío. Los TAG existentes nunca se sobrescriben.</x:v>
       </x:c>
     </x:row>
     <x:row r="55" ht="23" customHeight="1">
@@ -1072,44 +1071,44 @@
     </x:row>
     <x:row r="56" ht="23" customHeight="1">
       <x:c r="A56" s="5" t="str">
-        <x:v>En la ficha se mostrará un listado de componentes y la tabla de fabricantes de referencia con descripción y web. En las tarjetas del catálogo se mostrarán los nombres de esos fabricantes separados por coma. Las referencias comerciales no confirman el fabricante instalado.</x:v>
+        <x:v>En la ficha se mostrará un listado de componentes y fabricantes de referencia con descripción y web. En las tarjetas del catálogo se mostrarán los nombres de esos fabricantes separados por coma. Los filtros agrupan mayúsculas y espacios; filtrar por cualquier referencia devuelve el modelo una sola vez.</x:v>
       </x:c>
       <x:c r="B56" s="5" t="str">
-        <x:v>En la ficha se mostrará un listado de componentes y la tabla de fabricantes de referencia con descripción y web. En las tarjetas del catálogo se mostrarán los nombres de esos fabricantes separados por coma. Las referencias comerciales no confirman el fabricante instalado.</x:v>
+        <x:v>En la ficha se mostrará un listado de componentes y fabricantes de referencia con descripción y web. En las tarjetas del catálogo se mostrarán los nombres de esos fabricantes separados por coma. Los filtros agrupan mayúsculas y espacios; filtrar por cualquier referencia devuelve el modelo una sola vez.</x:v>
       </x:c>
       <x:c r="C56" s="5" t="str">
-        <x:v>En la ficha se mostrará un listado de componentes y la tabla de fabricantes de referencia con descripción y web. En las tarjetas del catálogo se mostrarán los nombres de esos fabricantes separados por coma. Las referencias comerciales no confirman el fabricante instalado.</x:v>
+        <x:v>En la ficha se mostrará un listado de componentes y fabricantes de referencia con descripción y web. En las tarjetas del catálogo se mostrarán los nombres de esos fabricantes separados por coma. Los filtros agrupan mayúsculas y espacios; filtrar por cualquier referencia devuelve el modelo una sola vez.</x:v>
       </x:c>
       <x:c r="D56" s="5" t="str">
-        <x:v>En la ficha se mostrará un listado de componentes y la tabla de fabricantes de referencia con descripción y web. En las tarjetas del catálogo se mostrarán los nombres de esos fabricantes separados por coma. Las referencias comerciales no confirman el fabricante instalado.</x:v>
+        <x:v>En la ficha se mostrará un listado de componentes y fabricantes de referencia con descripción y web. En las tarjetas del catálogo se mostrarán los nombres de esos fabricantes separados por coma. Los filtros agrupan mayúsculas y espacios; filtrar por cualquier referencia devuelve el modelo una sola vez.</x:v>
       </x:c>
     </x:row>
     <x:row r="57" ht="23" customHeight="1">
       <x:c r="A57" s="5" t="str">
-        <x:v>En la ficha se mostrará un listado de componentes y la tabla de fabricantes de referencia con descripción y web. En las tarjetas del catálogo se mostrarán los nombres de esos fabricantes separados por coma. Las referencias comerciales no confirman el fabricante instalado.</x:v>
+        <x:v>En la ficha se mostrará un listado de componentes y fabricantes de referencia con descripción y web. En las tarjetas del catálogo se mostrarán los nombres de esos fabricantes separados por coma. Los filtros agrupan mayúsculas y espacios; filtrar por cualquier referencia devuelve el modelo una sola vez.</x:v>
       </x:c>
       <x:c r="B57" s="5" t="str">
-        <x:v>En la ficha se mostrará un listado de componentes y la tabla de fabricantes de referencia con descripción y web. En las tarjetas del catálogo se mostrarán los nombres de esos fabricantes separados por coma. Las referencias comerciales no confirman el fabricante instalado.</x:v>
+        <x:v>En la ficha se mostrará un listado de componentes y fabricantes de referencia con descripción y web. En las tarjetas del catálogo se mostrarán los nombres de esos fabricantes separados por coma. Los filtros agrupan mayúsculas y espacios; filtrar por cualquier referencia devuelve el modelo una sola vez.</x:v>
       </x:c>
       <x:c r="C57" s="5" t="str">
-        <x:v>En la ficha se mostrará un listado de componentes y la tabla de fabricantes de referencia con descripción y web. En las tarjetas del catálogo se mostrarán los nombres de esos fabricantes separados por coma. Las referencias comerciales no confirman el fabricante instalado.</x:v>
+        <x:v>En la ficha se mostrará un listado de componentes y fabricantes de referencia con descripción y web. En las tarjetas del catálogo se mostrarán los nombres de esos fabricantes separados por coma. Los filtros agrupan mayúsculas y espacios; filtrar por cualquier referencia devuelve el modelo una sola vez.</x:v>
       </x:c>
       <x:c r="D57" s="5" t="str">
-        <x:v>En la ficha se mostrará un listado de componentes y la tabla de fabricantes de referencia con descripción y web. En las tarjetas del catálogo se mostrarán los nombres de esos fabricantes separados por coma. Las referencias comerciales no confirman el fabricante instalado.</x:v>
+        <x:v>En la ficha se mostrará un listado de componentes y fabricantes de referencia con descripción y web. En las tarjetas del catálogo se mostrarán los nombres de esos fabricantes separados por coma. Los filtros agrupan mayúsculas y espacios; filtrar por cualquier referencia devuelve el modelo una sola vez.</x:v>
       </x:c>
     </x:row>
     <x:row r="58" ht="23" customHeight="1">
       <x:c r="A58" s="5" t="str">
-        <x:v>En la ficha se mostrará un listado de componentes y la tabla de fabricantes de referencia con descripción y web. En las tarjetas del catálogo se mostrarán los nombres de esos fabricantes separados por coma. Las referencias comerciales no confirman el fabricante instalado.</x:v>
+        <x:v>En la ficha se mostrará un listado de componentes y fabricantes de referencia con descripción y web. En las tarjetas del catálogo se mostrarán los nombres de esos fabricantes separados por coma. Los filtros agrupan mayúsculas y espacios; filtrar por cualquier referencia devuelve el modelo una sola vez.</x:v>
       </x:c>
       <x:c r="B58" s="5" t="str">
-        <x:v>En la ficha se mostrará un listado de componentes y la tabla de fabricantes de referencia con descripción y web. En las tarjetas del catálogo se mostrarán los nombres de esos fabricantes separados por coma. Las referencias comerciales no confirman el fabricante instalado.</x:v>
+        <x:v>En la ficha se mostrará un listado de componentes y fabricantes de referencia con descripción y web. En las tarjetas del catálogo se mostrarán los nombres de esos fabricantes separados por coma. Los filtros agrupan mayúsculas y espacios; filtrar por cualquier referencia devuelve el modelo una sola vez.</x:v>
       </x:c>
       <x:c r="C58" s="5" t="str">
-        <x:v>En la ficha se mostrará un listado de componentes y la tabla de fabricantes de referencia con descripción y web. En las tarjetas del catálogo se mostrarán los nombres de esos fabricantes separados por coma. Las referencias comerciales no confirman el fabricante instalado.</x:v>
+        <x:v>En la ficha se mostrará un listado de componentes y fabricantes de referencia con descripción y web. En las tarjetas del catálogo se mostrarán los nombres de esos fabricantes separados por coma. Los filtros agrupan mayúsculas y espacios; filtrar por cualquier referencia devuelve el modelo una sola vez.</x:v>
       </x:c>
       <x:c r="D58" s="5" t="str">
-        <x:v>En la ficha se mostrará un listado de componentes y la tabla de fabricantes de referencia con descripción y web. En las tarjetas del catálogo se mostrarán los nombres de esos fabricantes separados por coma. Las referencias comerciales no confirman el fabricante instalado.</x:v>
+        <x:v>En la ficha se mostrará un listado de componentes y fabricantes de referencia con descripción y web. En las tarjetas del catálogo se mostrarán los nombres de esos fabricantes separados por coma. Los filtros agrupan mayúsculas y espacios; filtrar por cualquier referencia devuelve el modelo una sola vez.</x:v>
       </x:c>
     </x:row>
     <x:row r="59" ht="23" customHeight="1">
@@ -1174,8 +1173,7 @@
     <x:col min="3" max="3" width="16" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="48" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="48" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="32" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="48" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="48" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="32" customHeight="1">
@@ -1194,10 +1192,7 @@
       <x:c r="E1" s="23" t="str">
         <x:v>Tipo</x:v>
       </x:c>
-      <x:c r="F1" s="23" t="str">
-        <x:v>Fabricante / modelo</x:v>
-      </x:c>
-      <x:c r="G1" s="24" t="str">
+      <x:c r="F1" s="24" t="str">
         <x:v>Denominación de etapa</x:v>
       </x:c>
     </x:row>
@@ -1208,7 +1203,6 @@
       <x:c r="D2" s="16"/>
       <x:c r="E2" s="16"/>
       <x:c r="F2" s="16"/>
-      <x:c r="G2" s="16"/>
     </x:row>
     <x:row r="3" ht="25" customHeight="1">
       <x:c r="A3" s="16"/>
@@ -1217,7 +1211,6 @@
       <x:c r="D3" s="16"/>
       <x:c r="E3" s="16"/>
       <x:c r="F3" s="16"/>
-      <x:c r="G3" s="16"/>
     </x:row>
     <x:row r="4" ht="25" customHeight="1">
       <x:c r="A4" s="16"/>
@@ -1226,7 +1219,6 @@
       <x:c r="D4" s="16"/>
       <x:c r="E4" s="16"/>
       <x:c r="F4" s="16"/>
-      <x:c r="G4" s="16"/>
     </x:row>
     <x:row r="5" ht="25" customHeight="1">
       <x:c r="A5" s="16"/>
@@ -1235,7 +1227,6 @@
       <x:c r="D5" s="16"/>
       <x:c r="E5" s="16"/>
       <x:c r="F5" s="16"/>
-      <x:c r="G5" s="16"/>
     </x:row>
     <x:row r="6" ht="25" customHeight="1">
       <x:c r="A6" s="16"/>
@@ -1244,7 +1235,6 @@
       <x:c r="D6" s="16"/>
       <x:c r="E6" s="16"/>
       <x:c r="F6" s="16"/>
-      <x:c r="G6" s="16"/>
     </x:row>
     <x:row r="7" ht="25" customHeight="1">
       <x:c r="A7" s="16"/>
@@ -1253,7 +1243,6 @@
       <x:c r="D7" s="16"/>
       <x:c r="E7" s="16"/>
       <x:c r="F7" s="16"/>
-      <x:c r="G7" s="16"/>
     </x:row>
     <x:row r="8" ht="25" customHeight="1">
       <x:c r="A8" s="16"/>
@@ -1262,7 +1251,6 @@
       <x:c r="D8" s="16"/>
       <x:c r="E8" s="16"/>
       <x:c r="F8" s="16"/>
-      <x:c r="G8" s="16"/>
     </x:row>
     <x:row r="9" ht="25" customHeight="1">
       <x:c r="A9" s="16"/>
@@ -1271,7 +1259,6 @@
       <x:c r="D9" s="16"/>
       <x:c r="E9" s="16"/>
       <x:c r="F9" s="16"/>
-      <x:c r="G9" s="16"/>
     </x:row>
     <x:row r="10" ht="25" customHeight="1">
       <x:c r="A10" s="16"/>
@@ -1280,7 +1267,6 @@
       <x:c r="D10" s="16"/>
       <x:c r="E10" s="16"/>
       <x:c r="F10" s="16"/>
-      <x:c r="G10" s="16"/>
     </x:row>
     <x:row r="11" ht="25" customHeight="1">
       <x:c r="A11" s="16"/>
@@ -1289,7 +1275,6 @@
       <x:c r="D11" s="16"/>
       <x:c r="E11" s="16"/>
       <x:c r="F11" s="16"/>
-      <x:c r="G11" s="16"/>
     </x:row>
     <x:row r="12" ht="25" customHeight="1">
       <x:c r="A12" s="16"/>
@@ -1298,7 +1283,6 @@
       <x:c r="D12" s="16"/>
       <x:c r="E12" s="16"/>
       <x:c r="F12" s="16"/>
-      <x:c r="G12" s="16"/>
     </x:row>
     <x:row r="13" ht="25" customHeight="1">
       <x:c r="A13" s="16"/>
@@ -1307,7 +1291,6 @@
       <x:c r="D13" s="16"/>
       <x:c r="E13" s="16"/>
       <x:c r="F13" s="16"/>
-      <x:c r="G13" s="16"/>
     </x:row>
     <x:row r="14" ht="25" customHeight="1">
       <x:c r="A14" s="16"/>
@@ -1316,7 +1299,6 @@
       <x:c r="D14" s="16"/>
       <x:c r="E14" s="16"/>
       <x:c r="F14" s="16"/>
-      <x:c r="G14" s="16"/>
     </x:row>
     <x:row r="15" ht="25" customHeight="1">
       <x:c r="A15" s="16"/>
@@ -1325,7 +1307,6 @@
       <x:c r="D15" s="16"/>
       <x:c r="E15" s="16"/>
       <x:c r="F15" s="16"/>
-      <x:c r="G15" s="16"/>
     </x:row>
     <x:row r="16" ht="25" customHeight="1">
       <x:c r="A16" s="16"/>
@@ -1334,7 +1315,6 @@
       <x:c r="D16" s="16"/>
       <x:c r="E16" s="16"/>
       <x:c r="F16" s="16"/>
-      <x:c r="G16" s="16"/>
     </x:row>
     <x:row r="17" ht="25" customHeight="1">
       <x:c r="A17" s="16"/>
@@ -1343,7 +1323,6 @@
       <x:c r="D17" s="16"/>
       <x:c r="E17" s="16"/>
       <x:c r="F17" s="16"/>
-      <x:c r="G17" s="16"/>
     </x:row>
     <x:row r="18" ht="25" customHeight="1">
       <x:c r="A18" s="16"/>
@@ -1352,7 +1331,6 @@
       <x:c r="D18" s="16"/>
       <x:c r="E18" s="16"/>
       <x:c r="F18" s="16"/>
-      <x:c r="G18" s="16"/>
     </x:row>
     <x:row r="19" ht="25" customHeight="1">
       <x:c r="A19" s="16"/>
@@ -1361,7 +1339,6 @@
       <x:c r="D19" s="16"/>
       <x:c r="E19" s="16"/>
       <x:c r="F19" s="16"/>
-      <x:c r="G19" s="16"/>
     </x:row>
     <x:row r="20" ht="25" customHeight="1">
       <x:c r="A20" s="16"/>
@@ -1370,7 +1347,6 @@
       <x:c r="D20" s="16"/>
       <x:c r="E20" s="16"/>
       <x:c r="F20" s="16"/>
-      <x:c r="G20" s="16"/>
     </x:row>
     <x:row r="21" ht="25" customHeight="1">
       <x:c r="A21" s="16"/>
@@ -1379,7 +1355,6 @@
       <x:c r="D21" s="16"/>
       <x:c r="E21" s="16"/>
       <x:c r="F21" s="16"/>
-      <x:c r="G21" s="16"/>
     </x:row>
     <x:row r="22" ht="25" customHeight="1">
       <x:c r="A22" s="16"/>
@@ -1388,7 +1363,6 @@
       <x:c r="D22" s="16"/>
       <x:c r="E22" s="16"/>
       <x:c r="F22" s="16"/>
-      <x:c r="G22" s="16"/>
     </x:row>
     <x:row r="23" ht="25" customHeight="1">
       <x:c r="A23" s="16"/>
@@ -1397,7 +1371,6 @@
       <x:c r="D23" s="16"/>
       <x:c r="E23" s="16"/>
       <x:c r="F23" s="16"/>
-      <x:c r="G23" s="16"/>
     </x:row>
     <x:row r="24" ht="25" customHeight="1">
       <x:c r="A24" s="16"/>
@@ -1406,7 +1379,6 @@
       <x:c r="D24" s="16"/>
       <x:c r="E24" s="16"/>
       <x:c r="F24" s="16"/>
-      <x:c r="G24" s="16"/>
     </x:row>
     <x:row r="25" ht="25" customHeight="1">
       <x:c r="A25" s="16"/>
@@ -1415,7 +1387,6 @@
       <x:c r="D25" s="16"/>
       <x:c r="E25" s="16"/>
       <x:c r="F25" s="16"/>
-      <x:c r="G25" s="16"/>
     </x:row>
     <x:row r="26" ht="25" customHeight="1">
       <x:c r="A26" s="16"/>
@@ -1424,7 +1395,6 @@
       <x:c r="D26" s="16"/>
       <x:c r="E26" s="16"/>
       <x:c r="F26" s="16"/>
-      <x:c r="G26" s="16"/>
     </x:row>
     <x:row r="27" ht="25" customHeight="1">
       <x:c r="A27" s="16"/>
@@ -1433,7 +1403,6 @@
       <x:c r="D27" s="16"/>
       <x:c r="E27" s="16"/>
       <x:c r="F27" s="16"/>
-      <x:c r="G27" s="16"/>
     </x:row>
     <x:row r="28" ht="25" customHeight="1">
       <x:c r="A28" s="16"/>
@@ -1442,7 +1411,6 @@
       <x:c r="D28" s="16"/>
       <x:c r="E28" s="16"/>
       <x:c r="F28" s="16"/>
-      <x:c r="G28" s="16"/>
     </x:row>
     <x:row r="29" ht="25" customHeight="1">
       <x:c r="A29" s="16"/>
@@ -1451,7 +1419,6 @@
       <x:c r="D29" s="16"/>
       <x:c r="E29" s="16"/>
       <x:c r="F29" s="16"/>
-      <x:c r="G29" s="16"/>
     </x:row>
     <x:row r="30" ht="25" customHeight="1">
       <x:c r="A30" s="16"/>
@@ -1460,7 +1427,6 @@
       <x:c r="D30" s="16"/>
       <x:c r="E30" s="16"/>
       <x:c r="F30" s="16"/>
-      <x:c r="G30" s="16"/>
     </x:row>
     <x:row r="31" ht="25" customHeight="1">
       <x:c r="A31" s="16"/>
@@ -1469,7 +1435,6 @@
       <x:c r="D31" s="16"/>
       <x:c r="E31" s="16"/>
       <x:c r="F31" s="16"/>
-      <x:c r="G31" s="16"/>
     </x:row>
     <x:row r="32" ht="25" customHeight="1">
       <x:c r="A32" s="16"/>
@@ -1478,7 +1443,6 @@
       <x:c r="D32" s="16"/>
       <x:c r="E32" s="16"/>
       <x:c r="F32" s="16"/>
-      <x:c r="G32" s="16"/>
     </x:row>
     <x:row r="33" ht="25" customHeight="1">
       <x:c r="A33" s="16"/>
@@ -1487,7 +1451,6 @@
       <x:c r="D33" s="16"/>
       <x:c r="E33" s="16"/>
       <x:c r="F33" s="16"/>
-      <x:c r="G33" s="16"/>
     </x:row>
     <x:row r="34" ht="25" customHeight="1">
       <x:c r="A34" s="16"/>
@@ -1496,7 +1459,6 @@
       <x:c r="D34" s="16"/>
       <x:c r="E34" s="16"/>
       <x:c r="F34" s="16"/>
-      <x:c r="G34" s="16"/>
     </x:row>
     <x:row r="35" ht="25" customHeight="1">
       <x:c r="A35" s="16"/>
@@ -1505,7 +1467,6 @@
       <x:c r="D35" s="16"/>
       <x:c r="E35" s="16"/>
       <x:c r="F35" s="16"/>
-      <x:c r="G35" s="16"/>
     </x:row>
     <x:row r="36" ht="25" customHeight="1">
       <x:c r="A36" s="16"/>
@@ -1514,7 +1475,6 @@
       <x:c r="D36" s="16"/>
       <x:c r="E36" s="16"/>
       <x:c r="F36" s="16"/>
-      <x:c r="G36" s="16"/>
     </x:row>
     <x:row r="37" ht="25" customHeight="1">
       <x:c r="A37" s="16"/>
@@ -1523,7 +1483,6 @@
       <x:c r="D37" s="16"/>
       <x:c r="E37" s="16"/>
       <x:c r="F37" s="16"/>
-      <x:c r="G37" s="16"/>
     </x:row>
     <x:row r="38" ht="25" customHeight="1">
       <x:c r="A38" s="16"/>
@@ -1532,7 +1491,6 @@
       <x:c r="D38" s="16"/>
       <x:c r="E38" s="16"/>
       <x:c r="F38" s="16"/>
-      <x:c r="G38" s="16"/>
     </x:row>
     <x:row r="39" ht="25" customHeight="1">
       <x:c r="A39" s="16"/>
@@ -1541,7 +1499,6 @@
       <x:c r="D39" s="16"/>
       <x:c r="E39" s="16"/>
       <x:c r="F39" s="16"/>
-      <x:c r="G39" s="16"/>
     </x:row>
     <x:row r="40" ht="25" customHeight="1">
       <x:c r="A40" s="16"/>
@@ -1550,7 +1507,6 @@
       <x:c r="D40" s="16"/>
       <x:c r="E40" s="16"/>
       <x:c r="F40" s="16"/>
-      <x:c r="G40" s="16"/>
     </x:row>
     <x:row r="41" ht="25" customHeight="1">
       <x:c r="A41" s="16"/>
@@ -1559,7 +1515,6 @@
       <x:c r="D41" s="16"/>
       <x:c r="E41" s="16"/>
       <x:c r="F41" s="16"/>
-      <x:c r="G41" s="16"/>
     </x:row>
     <x:row r="42" ht="25" customHeight="1">
       <x:c r="A42" s="16"/>
@@ -1568,7 +1523,6 @@
       <x:c r="D42" s="16"/>
       <x:c r="E42" s="16"/>
       <x:c r="F42" s="16"/>
-      <x:c r="G42" s="16"/>
     </x:row>
     <x:row r="43" ht="25" customHeight="1">
       <x:c r="A43" s="16"/>
@@ -1577,7 +1531,6 @@
       <x:c r="D43" s="16"/>
       <x:c r="E43" s="16"/>
       <x:c r="F43" s="16"/>
-      <x:c r="G43" s="16"/>
     </x:row>
     <x:row r="44" ht="25" customHeight="1">
       <x:c r="A44" s="16"/>
@@ -1586,7 +1539,6 @@
       <x:c r="D44" s="16"/>
       <x:c r="E44" s="16"/>
       <x:c r="F44" s="16"/>
-      <x:c r="G44" s="16"/>
     </x:row>
     <x:row r="45" ht="25" customHeight="1">
       <x:c r="A45" s="16"/>
@@ -1595,7 +1547,6 @@
       <x:c r="D45" s="16"/>
       <x:c r="E45" s="16"/>
       <x:c r="F45" s="16"/>
-      <x:c r="G45" s="16"/>
     </x:row>
     <x:row r="46" ht="25" customHeight="1">
       <x:c r="A46" s="16"/>
@@ -1604,7 +1555,6 @@
       <x:c r="D46" s="16"/>
       <x:c r="E46" s="16"/>
       <x:c r="F46" s="16"/>
-      <x:c r="G46" s="16"/>
     </x:row>
     <x:row r="47" ht="25" customHeight="1">
       <x:c r="A47" s="16"/>
@@ -1613,7 +1563,6 @@
       <x:c r="D47" s="16"/>
       <x:c r="E47" s="16"/>
       <x:c r="F47" s="16"/>
-      <x:c r="G47" s="16"/>
     </x:row>
     <x:row r="48" ht="25" customHeight="1">
       <x:c r="A48" s="16"/>
@@ -1622,7 +1571,6 @@
       <x:c r="D48" s="16"/>
       <x:c r="E48" s="16"/>
       <x:c r="F48" s="16"/>
-      <x:c r="G48" s="16"/>
     </x:row>
     <x:row r="49" ht="25" customHeight="1">
       <x:c r="A49" s="16"/>
@@ -1631,7 +1579,6 @@
       <x:c r="D49" s="16"/>
       <x:c r="E49" s="16"/>
       <x:c r="F49" s="16"/>
-      <x:c r="G49" s="16"/>
     </x:row>
     <x:row r="50" ht="25" customHeight="1">
       <x:c r="A50" s="16"/>
@@ -1640,7 +1587,6 @@
       <x:c r="D50" s="16"/>
       <x:c r="E50" s="16"/>
       <x:c r="F50" s="16"/>
-      <x:c r="G50" s="16"/>
     </x:row>
     <x:row r="51" ht="25" customHeight="1">
       <x:c r="A51" s="16"/>
@@ -1649,7 +1595,6 @@
       <x:c r="D51" s="16"/>
       <x:c r="E51" s="16"/>
       <x:c r="F51" s="16"/>
-      <x:c r="G51" s="16"/>
     </x:row>
     <x:row r="52" ht="25" customHeight="1">
       <x:c r="A52" s="16"/>
@@ -1658,7 +1603,6 @@
       <x:c r="D52" s="16"/>
       <x:c r="E52" s="16"/>
       <x:c r="F52" s="16"/>
-      <x:c r="G52" s="16"/>
     </x:row>
     <x:row r="53" ht="25" customHeight="1">
       <x:c r="A53" s="16"/>
@@ -1667,7 +1611,6 @@
       <x:c r="D53" s="16"/>
       <x:c r="E53" s="16"/>
       <x:c r="F53" s="16"/>
-      <x:c r="G53" s="16"/>
     </x:row>
     <x:row r="54" ht="25" customHeight="1">
       <x:c r="A54" s="16"/>
@@ -1676,7 +1619,6 @@
       <x:c r="D54" s="16"/>
       <x:c r="E54" s="16"/>
       <x:c r="F54" s="16"/>
-      <x:c r="G54" s="16"/>
     </x:row>
     <x:row r="55" ht="25" customHeight="1">
       <x:c r="A55" s="16"/>
@@ -1685,7 +1627,6 @@
       <x:c r="D55" s="16"/>
       <x:c r="E55" s="16"/>
       <x:c r="F55" s="16"/>
-      <x:c r="G55" s="16"/>
     </x:row>
     <x:row r="56" ht="25" customHeight="1">
       <x:c r="A56" s="16"/>
@@ -1694,7 +1635,6 @@
       <x:c r="D56" s="16"/>
       <x:c r="E56" s="16"/>
       <x:c r="F56" s="16"/>
-      <x:c r="G56" s="16"/>
     </x:row>
     <x:row r="57" ht="25" customHeight="1">
       <x:c r="A57" s="16"/>
@@ -1703,7 +1643,6 @@
       <x:c r="D57" s="16"/>
       <x:c r="E57" s="16"/>
       <x:c r="F57" s="16"/>
-      <x:c r="G57" s="16"/>
     </x:row>
     <x:row r="58" ht="25" customHeight="1">
       <x:c r="A58" s="16"/>
@@ -1712,7 +1651,6 @@
       <x:c r="D58" s="16"/>
       <x:c r="E58" s="16"/>
       <x:c r="F58" s="16"/>
-      <x:c r="G58" s="16"/>
     </x:row>
     <x:row r="59" ht="25" customHeight="1">
       <x:c r="A59" s="16"/>
@@ -1721,7 +1659,6 @@
       <x:c r="D59" s="16"/>
       <x:c r="E59" s="16"/>
       <x:c r="F59" s="16"/>
-      <x:c r="G59" s="16"/>
     </x:row>
     <x:row r="60" ht="25" customHeight="1">
       <x:c r="A60" s="16"/>
@@ -1730,7 +1667,6 @@
       <x:c r="D60" s="16"/>
       <x:c r="E60" s="16"/>
       <x:c r="F60" s="16"/>
-      <x:c r="G60" s="16"/>
     </x:row>
     <x:row r="61" ht="25" customHeight="1">
       <x:c r="A61" s="16"/>
@@ -1739,7 +1675,6 @@
       <x:c r="D61" s="16"/>
       <x:c r="E61" s="16"/>
       <x:c r="F61" s="16"/>
-      <x:c r="G61" s="16"/>
     </x:row>
     <x:row r="62" ht="25" customHeight="1">
       <x:c r="A62" s="16"/>
@@ -1748,7 +1683,6 @@
       <x:c r="D62" s="16"/>
       <x:c r="E62" s="16"/>
       <x:c r="F62" s="16"/>
-      <x:c r="G62" s="16"/>
     </x:row>
     <x:row r="63" ht="25" customHeight="1">
       <x:c r="A63" s="16"/>
@@ -1757,7 +1691,6 @@
       <x:c r="D63" s="16"/>
       <x:c r="E63" s="16"/>
       <x:c r="F63" s="16"/>
-      <x:c r="G63" s="16"/>
     </x:row>
     <x:row r="64" ht="25" customHeight="1">
       <x:c r="A64" s="16"/>
@@ -1766,7 +1699,6 @@
       <x:c r="D64" s="16"/>
       <x:c r="E64" s="16"/>
       <x:c r="F64" s="16"/>
-      <x:c r="G64" s="16"/>
     </x:row>
     <x:row r="65" ht="25" customHeight="1">
       <x:c r="A65" s="16"/>
@@ -1775,7 +1707,6 @@
       <x:c r="D65" s="16"/>
       <x:c r="E65" s="16"/>
       <x:c r="F65" s="16"/>
-      <x:c r="G65" s="16"/>
     </x:row>
     <x:row r="66" ht="25" customHeight="1">
       <x:c r="A66" s="16"/>
@@ -1784,7 +1715,6 @@
       <x:c r="D66" s="16"/>
       <x:c r="E66" s="16"/>
       <x:c r="F66" s="16"/>
-      <x:c r="G66" s="16"/>
     </x:row>
     <x:row r="67" ht="25" customHeight="1">
       <x:c r="A67" s="16"/>
@@ -1793,7 +1723,6 @@
       <x:c r="D67" s="16"/>
       <x:c r="E67" s="16"/>
       <x:c r="F67" s="16"/>
-      <x:c r="G67" s="16"/>
     </x:row>
     <x:row r="68" ht="25" customHeight="1">
       <x:c r="A68" s="16"/>
@@ -1802,7 +1731,6 @@
       <x:c r="D68" s="16"/>
       <x:c r="E68" s="16"/>
       <x:c r="F68" s="16"/>
-      <x:c r="G68" s="16"/>
     </x:row>
     <x:row r="69" ht="25" customHeight="1">
       <x:c r="A69" s="16"/>
@@ -1811,7 +1739,6 @@
       <x:c r="D69" s="16"/>
       <x:c r="E69" s="16"/>
       <x:c r="F69" s="16"/>
-      <x:c r="G69" s="16"/>
     </x:row>
     <x:row r="70" ht="25" customHeight="1">
       <x:c r="A70" s="16"/>
@@ -1820,7 +1747,6 @@
       <x:c r="D70" s="16"/>
       <x:c r="E70" s="16"/>
       <x:c r="F70" s="16"/>
-      <x:c r="G70" s="16"/>
     </x:row>
     <x:row r="71" ht="25" customHeight="1">
       <x:c r="A71" s="16"/>
@@ -1829,7 +1755,6 @@
       <x:c r="D71" s="16"/>
       <x:c r="E71" s="16"/>
       <x:c r="F71" s="16"/>
-      <x:c r="G71" s="16"/>
     </x:row>
     <x:row r="72" ht="25" customHeight="1">
       <x:c r="A72" s="16"/>
@@ -1838,7 +1763,6 @@
       <x:c r="D72" s="16"/>
       <x:c r="E72" s="16"/>
       <x:c r="F72" s="16"/>
-      <x:c r="G72" s="16"/>
     </x:row>
     <x:row r="73" ht="25" customHeight="1">
       <x:c r="A73" s="16"/>
@@ -1847,7 +1771,6 @@
       <x:c r="D73" s="16"/>
       <x:c r="E73" s="16"/>
       <x:c r="F73" s="16"/>
-      <x:c r="G73" s="16"/>
     </x:row>
     <x:row r="74" ht="25" customHeight="1">
       <x:c r="A74" s="16"/>
@@ -1856,7 +1779,6 @@
       <x:c r="D74" s="16"/>
       <x:c r="E74" s="16"/>
       <x:c r="F74" s="16"/>
-      <x:c r="G74" s="16"/>
     </x:row>
     <x:row r="75" ht="25" customHeight="1">
       <x:c r="A75" s="16"/>
@@ -1865,7 +1787,6 @@
       <x:c r="D75" s="16"/>
       <x:c r="E75" s="16"/>
       <x:c r="F75" s="16"/>
-      <x:c r="G75" s="16"/>
     </x:row>
     <x:row r="76" ht="25" customHeight="1">
       <x:c r="A76" s="16"/>
@@ -1874,7 +1795,6 @@
       <x:c r="D76" s="16"/>
       <x:c r="E76" s="16"/>
       <x:c r="F76" s="16"/>
-      <x:c r="G76" s="16"/>
     </x:row>
     <x:row r="77" ht="25" customHeight="1">
       <x:c r="A77" s="16"/>
@@ -1883,7 +1803,6 @@
       <x:c r="D77" s="16"/>
       <x:c r="E77" s="16"/>
       <x:c r="F77" s="16"/>
-      <x:c r="G77" s="16"/>
     </x:row>
     <x:row r="78" ht="25" customHeight="1">
       <x:c r="A78" s="16"/>
@@ -1892,7 +1811,6 @@
       <x:c r="D78" s="16"/>
       <x:c r="E78" s="16"/>
       <x:c r="F78" s="16"/>
-      <x:c r="G78" s="16"/>
     </x:row>
     <x:row r="79" ht="25" customHeight="1">
       <x:c r="A79" s="16"/>
@@ -1901,7 +1819,6 @@
       <x:c r="D79" s="16"/>
       <x:c r="E79" s="16"/>
       <x:c r="F79" s="16"/>
-      <x:c r="G79" s="16"/>
     </x:row>
     <x:row r="80" ht="25" customHeight="1">
       <x:c r="A80" s="16"/>
@@ -1910,7 +1827,6 @@
       <x:c r="D80" s="16"/>
       <x:c r="E80" s="16"/>
       <x:c r="F80" s="16"/>
-      <x:c r="G80" s="16"/>
     </x:row>
     <x:row r="81" ht="25" customHeight="1">
       <x:c r="A81" s="16"/>
@@ -1919,7 +1835,6 @@
       <x:c r="D81" s="16"/>
       <x:c r="E81" s="16"/>
       <x:c r="F81" s="16"/>
-      <x:c r="G81" s="16"/>
     </x:row>
     <x:row r="82" ht="25" customHeight="1">
       <x:c r="A82" s="16"/>
@@ -1928,7 +1843,6 @@
       <x:c r="D82" s="16"/>
       <x:c r="E82" s="16"/>
       <x:c r="F82" s="16"/>
-      <x:c r="G82" s="16"/>
     </x:row>
     <x:row r="83" ht="25" customHeight="1">
       <x:c r="A83" s="16"/>
@@ -1937,7 +1851,6 @@
       <x:c r="D83" s="16"/>
       <x:c r="E83" s="16"/>
       <x:c r="F83" s="16"/>
-      <x:c r="G83" s="16"/>
     </x:row>
     <x:row r="84" ht="25" customHeight="1">
       <x:c r="A84" s="16"/>
@@ -1946,7 +1859,6 @@
       <x:c r="D84" s="16"/>
       <x:c r="E84" s="16"/>
       <x:c r="F84" s="16"/>
-      <x:c r="G84" s="16"/>
     </x:row>
     <x:row r="85" ht="25" customHeight="1">
       <x:c r="A85" s="16"/>
@@ -1955,7 +1867,6 @@
       <x:c r="D85" s="16"/>
       <x:c r="E85" s="16"/>
       <x:c r="F85" s="16"/>
-      <x:c r="G85" s="16"/>
     </x:row>
     <x:row r="86" ht="25" customHeight="1">
       <x:c r="A86" s="16"/>
@@ -1964,7 +1875,6 @@
       <x:c r="D86" s="16"/>
       <x:c r="E86" s="16"/>
       <x:c r="F86" s="16"/>
-      <x:c r="G86" s="16"/>
     </x:row>
     <x:row r="87" ht="25" customHeight="1">
       <x:c r="A87" s="16"/>
@@ -1973,7 +1883,6 @@
       <x:c r="D87" s="16"/>
       <x:c r="E87" s="16"/>
       <x:c r="F87" s="16"/>
-      <x:c r="G87" s="16"/>
     </x:row>
     <x:row r="88" ht="25" customHeight="1">
       <x:c r="A88" s="16"/>
@@ -1982,7 +1891,6 @@
       <x:c r="D88" s="16"/>
       <x:c r="E88" s="16"/>
       <x:c r="F88" s="16"/>
-      <x:c r="G88" s="16"/>
     </x:row>
     <x:row r="89" ht="25" customHeight="1">
       <x:c r="A89" s="16"/>
@@ -1991,7 +1899,6 @@
       <x:c r="D89" s="16"/>
       <x:c r="E89" s="16"/>
       <x:c r="F89" s="16"/>
-      <x:c r="G89" s="16"/>
     </x:row>
     <x:row r="90" ht="25" customHeight="1">
       <x:c r="A90" s="16"/>
@@ -2000,7 +1907,6 @@
       <x:c r="D90" s="16"/>
       <x:c r="E90" s="16"/>
       <x:c r="F90" s="16"/>
-      <x:c r="G90" s="16"/>
     </x:row>
     <x:row r="91" ht="25" customHeight="1">
       <x:c r="A91" s="16"/>
@@ -2009,7 +1915,6 @@
       <x:c r="D91" s="16"/>
       <x:c r="E91" s="16"/>
       <x:c r="F91" s="16"/>
-      <x:c r="G91" s="16"/>
     </x:row>
     <x:row r="92" ht="25" customHeight="1">
       <x:c r="A92" s="16"/>
@@ -2018,7 +1923,6 @@
       <x:c r="D92" s="16"/>
       <x:c r="E92" s="16"/>
       <x:c r="F92" s="16"/>
-      <x:c r="G92" s="16"/>
     </x:row>
     <x:row r="93" ht="25" customHeight="1">
       <x:c r="A93" s="16"/>
@@ -2027,7 +1931,6 @@
       <x:c r="D93" s="16"/>
       <x:c r="E93" s="16"/>
       <x:c r="F93" s="16"/>
-      <x:c r="G93" s="16"/>
     </x:row>
     <x:row r="94" ht="25" customHeight="1">
       <x:c r="A94" s="16"/>
@@ -2036,7 +1939,6 @@
       <x:c r="D94" s="16"/>
       <x:c r="E94" s="16"/>
       <x:c r="F94" s="16"/>
-      <x:c r="G94" s="16"/>
     </x:row>
     <x:row r="95" ht="25" customHeight="1">
       <x:c r="A95" s="16"/>
@@ -2045,7 +1947,6 @@
       <x:c r="D95" s="16"/>
       <x:c r="E95" s="16"/>
       <x:c r="F95" s="16"/>
-      <x:c r="G95" s="16"/>
     </x:row>
     <x:row r="96" ht="25" customHeight="1">
       <x:c r="A96" s="16"/>
@@ -2054,7 +1955,6 @@
       <x:c r="D96" s="16"/>
       <x:c r="E96" s="16"/>
       <x:c r="F96" s="16"/>
-      <x:c r="G96" s="16"/>
     </x:row>
     <x:row r="97" ht="25" customHeight="1">
       <x:c r="A97" s="16"/>
@@ -2063,7 +1963,6 @@
       <x:c r="D97" s="16"/>
       <x:c r="E97" s="16"/>
       <x:c r="F97" s="16"/>
-      <x:c r="G97" s="16"/>
     </x:row>
     <x:row r="98" ht="25" customHeight="1">
       <x:c r="A98" s="16"/>
@@ -2072,7 +1971,6 @@
       <x:c r="D98" s="16"/>
       <x:c r="E98" s="16"/>
       <x:c r="F98" s="16"/>
-      <x:c r="G98" s="16"/>
     </x:row>
     <x:row r="99" ht="25" customHeight="1">
       <x:c r="A99" s="16"/>
@@ -2081,7 +1979,6 @@
       <x:c r="D99" s="16"/>
       <x:c r="E99" s="16"/>
       <x:c r="F99" s="16"/>
-      <x:c r="G99" s="16"/>
     </x:row>
     <x:row r="100" ht="25" customHeight="1">
       <x:c r="A100" s="16"/>
@@ -2090,7 +1987,6 @@
       <x:c r="D100" s="16"/>
       <x:c r="E100" s="16"/>
       <x:c r="F100" s="16"/>
-      <x:c r="G100" s="16"/>
     </x:row>
     <x:row r="101" ht="25" customHeight="1">
       <x:c r="A101" s="16"/>
@@ -2099,7 +1995,6 @@
       <x:c r="D101" s="16"/>
       <x:c r="E101" s="16"/>
       <x:c r="F101" s="16"/>
-      <x:c r="G101" s="16"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
@@ -2109,7 +2004,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rfb77120cc35d4eb8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R79488564a3764172"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2565,7 +2460,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5de493a66884779"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc57836e6986b4b78"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2989,7 +2884,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra851cbc372014af1"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7a6a7d494443453c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3621,7 +3516,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb4157851b7be4fa6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb34029405b6a4132"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4253,7 +4148,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R414609714c204d8d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4550883c374b40a7"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>